<commit_message>
Updated Uploads Page & added more subjects
</commit_message>
<xml_diff>
--- a/RESULTS/2025/CLASS/SS3/English_language/results.xlsx
+++ b/RESULTS/2025/CLASS/SS3/English_language/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,6 +511,52 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>2025-12-12 22:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sulaiman Nazif</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>std389</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SS3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ENGLISH</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>87</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2025-12-12 23:11</t>
         </is>
       </c>
     </row>

</xml_diff>